<commit_message>
Atualiza Parciais da Rodada 7
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -55,12 +55,12 @@
     <t>Bandoleros FCS</t>
   </si>
   <si>
+    <t>JV5 Tricolor Gaúcho</t>
+  </si>
+  <si>
     <t>LISI GREMISTA</t>
   </si>
   <si>
-    <t>JV5 Tricolor Gaúcho</t>
-  </si>
-  <si>
     <t>Mau Humor F.C.</t>
   </si>
   <si>
@@ -82,15 +82,15 @@
     <t>Grupo K</t>
   </si>
   <si>
+    <t>Fedato Futebol Clube</t>
+  </si>
+  <si>
+    <t>TORRESMO COM PINGA PRO26.1</t>
+  </si>
+  <si>
     <t>TEAM LOPES 99</t>
   </si>
   <si>
-    <t>Fedato Futebol Clube</t>
-  </si>
-  <si>
-    <t>TORRESMO COM PINGA PRO26.1</t>
-  </si>
-  <si>
     <t>DM Studio</t>
   </si>
   <si>
@@ -100,10 +100,10 @@
     <t>Texas Club 2026</t>
   </si>
   <si>
+    <t>lsauer fc</t>
+  </si>
+  <si>
     <t>KillerColorado</t>
-  </si>
-  <si>
-    <t>lsauer fc</t>
   </si>
   <si>
     <t>Tabajara de Inhaua PB1</t>
@@ -507,10 +507,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -519,13 +519,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>527.3896484375</v>
+        <v>573.1596484375</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>23.67</v>
       </c>
       <c r="I2">
-        <v>527.3896484375</v>
+        <v>549.4896484375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -539,10 +539,10 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -551,13 +551,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>447.829345703125</v>
+        <v>476.689921875</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>30.67</v>
       </c>
       <c r="I3">
-        <v>447.829345703125</v>
+        <v>446.019921875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -580,16 +580,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>445.919921875</v>
+        <v>478.499345703125</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>30.77</v>
       </c>
       <c r="I4">
-        <v>445.919921875</v>
+        <v>447.729345703125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -612,16 +612,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>439.99951171875</v>
+        <v>463.66951171875</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>45.77</v>
       </c>
       <c r="I5">
-        <v>439.99951171875</v>
+        <v>417.89951171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -677,10 +677,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -689,13 +689,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>490.669921875</v>
+        <v>533.839921875</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>35.87</v>
       </c>
       <c r="I2">
-        <v>490.669921875</v>
+        <v>497.969921875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -709,10 +709,10 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -721,13 +721,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>478.1298828125</v>
+        <v>523.9998828125</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>35.8</v>
       </c>
       <c r="I3">
-        <v>478.1298828125</v>
+        <v>488.1998828125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -750,16 +750,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>442.719970703125</v>
+        <v>478.589970703125</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>43.17</v>
       </c>
       <c r="I4">
-        <v>442.719970703125</v>
+        <v>435.419970703125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>426.980224609375</v>
+        <v>462.780224609375</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>45.87</v>
       </c>
       <c r="I5">
-        <v>426.980224609375</v>
+        <v>416.910224609375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -847,10 +847,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>481.18994140625</v>
+        <v>544.5295703125</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>25.77</v>
       </c>
       <c r="I2">
-        <v>481.18994140625</v>
+        <v>518.7595703125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -879,10 +879,10 @@
         <v>22</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -891,13 +891,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>474.5595703125</v>
+        <v>507.279375</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>37.57</v>
       </c>
       <c r="I3">
-        <v>474.5595703125</v>
+        <v>469.709375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -920,16 +920,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>466.609375</v>
+        <v>518.7599414062501</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>40.67</v>
       </c>
       <c r="I4">
-        <v>466.609375</v>
+        <v>478.08994140625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>436.039794921875</v>
+        <v>461.809794921875</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>69.97</v>
       </c>
       <c r="I5">
-        <v>436.039794921875</v>
+        <v>391.839794921875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1017,10 +1017,10 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>497.169921875</v>
+        <v>540.339921875</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>39.17</v>
       </c>
       <c r="I2">
-        <v>497.169921875</v>
+        <v>501.1699218749999</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1049,10 +1049,10 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1061,13 +1061,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>485.85009765625</v>
+        <v>517.580205078125</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>27.4</v>
       </c>
       <c r="I3">
-        <v>485.85009765625</v>
+        <v>490.180205078125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>472.210205078125</v>
+        <v>513.25009765625</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>45.37</v>
       </c>
       <c r="I4">
-        <v>472.210205078125</v>
+        <v>467.88009765625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1122,16 +1122,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>443.6298828125</v>
+        <v>482.7998828125</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>43.17</v>
       </c>
       <c r="I5">
-        <v>443.6298828125</v>
+        <v>439.6298828125</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Resultado Final da Rodada 7
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -73,40 +73,40 @@
     <t>Dom Camillo68</t>
   </si>
   <si>
+    <t>Tatols Beants F.C</t>
+  </si>
+  <si>
     <t>A Lenda Super Vasco F.c</t>
   </si>
   <si>
-    <t>Tatols Beants F.C</t>
-  </si>
-  <si>
     <t>Grupo K</t>
   </si>
   <si>
     <t>Fedato Futebol Clube</t>
   </si>
   <si>
+    <t>TEAM LOPES 99</t>
+  </si>
+  <si>
     <t>TORRESMO COM PINGA PRO26.1</t>
   </si>
   <si>
-    <t>TEAM LOPES 99</t>
-  </si>
-  <si>
     <t>DM Studio</t>
   </si>
   <si>
     <t>Grupo L</t>
   </si>
   <si>
+    <t>lsauer fc</t>
+  </si>
+  <si>
+    <t>Tabajara de Inhaua PB1</t>
+  </si>
+  <si>
     <t>Texas Club 2026</t>
   </si>
   <si>
-    <t>lsauer fc</t>
-  </si>
-  <si>
     <t>KillerColorado</t>
-  </si>
-  <si>
-    <t>Tabajara de Inhaua PB1</t>
   </si>
 </sst>
 </file>
@@ -519,13 +519,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>573.1596484375</v>
+        <v>609.759765625</v>
       </c>
       <c r="H2">
-        <v>23.67</v>
+        <v>79.919921875</v>
       </c>
       <c r="I2">
-        <v>549.4896484375</v>
+        <v>529.83984375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -551,13 +551,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>476.689921875</v>
+        <v>522.98974609375</v>
       </c>
       <c r="H3">
-        <v>30.67</v>
+        <v>76.97021484375</v>
       </c>
       <c r="I3">
-        <v>446.019921875</v>
+        <v>446.01953125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>478.499345703125</v>
+        <v>524.799560546875</v>
       </c>
       <c r="H4">
-        <v>30.77</v>
+        <v>77.06982421875</v>
       </c>
       <c r="I4">
-        <v>447.729345703125</v>
+        <v>447.729736328125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -615,13 +615,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>463.66951171875</v>
+        <v>519.91943359375</v>
       </c>
       <c r="H5">
-        <v>45.77</v>
+        <v>82.3701171875</v>
       </c>
       <c r="I5">
-        <v>417.89951171875</v>
+        <v>437.54931640625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -689,13 +689,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>533.839921875</v>
+        <v>576.64013671875</v>
       </c>
       <c r="H2">
-        <v>35.87</v>
+        <v>50.570068359375</v>
       </c>
       <c r="I2">
-        <v>497.969921875</v>
+        <v>526.070068359375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -721,13 +721,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>523.9998828125</v>
+        <v>565.25</v>
       </c>
       <c r="H3">
-        <v>35.8</v>
+        <v>87.009765625</v>
       </c>
       <c r="I3">
-        <v>488.1998828125</v>
+        <v>478.240234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -753,13 +753,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>478.589970703125</v>
+        <v>513.989990234375</v>
       </c>
       <c r="H4">
-        <v>43.17</v>
+        <v>87.1201171875</v>
       </c>
       <c r="I4">
-        <v>435.419970703125</v>
+        <v>426.869873046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -785,13 +785,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>462.780224609375</v>
+        <v>493.2900390625</v>
       </c>
       <c r="H5">
-        <v>45.87</v>
+        <v>85.97021484375</v>
       </c>
       <c r="I5">
-        <v>416.910224609375</v>
+        <v>407.31982421875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>544.5295703125</v>
+        <v>580.4296875</v>
       </c>
       <c r="H2">
-        <v>25.77</v>
+        <v>72.1201171875</v>
       </c>
       <c r="I2">
-        <v>518.7595703125</v>
+        <v>508.3095703125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -891,13 +891,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>507.279375</v>
+        <v>552.56005859375</v>
       </c>
       <c r="H3">
-        <v>37.57</v>
+        <v>70.47021484375</v>
       </c>
       <c r="I3">
-        <v>469.709375</v>
+        <v>482.08984375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>518.7599414062501</v>
+        <v>537.07958984375</v>
       </c>
       <c r="H4">
-        <v>40.67</v>
+        <v>71.3701171875</v>
       </c>
       <c r="I4">
-        <v>478.08994140625</v>
+        <v>465.70947265625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -955,13 +955,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>461.809794921875</v>
+        <v>508.159912109375</v>
       </c>
       <c r="H5">
-        <v>69.97</v>
+        <v>105.8701171875</v>
       </c>
       <c r="I5">
-        <v>391.839794921875</v>
+        <v>402.289794921875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>540.339921875</v>
+        <v>553.780029296875</v>
       </c>
       <c r="H2">
-        <v>39.17</v>
+        <v>73.81982421875</v>
       </c>
       <c r="I2">
-        <v>501.1699218749999</v>
+        <v>479.960205078125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1061,13 +1061,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>517.580205078125</v>
+        <v>523.10009765625</v>
       </c>
       <c r="H3">
-        <v>27.4</v>
+        <v>76.97021484375</v>
       </c>
       <c r="I3">
-        <v>490.180205078125</v>
+        <v>446.1298828125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1093,13 +1093,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>513.25009765625</v>
+        <v>574.14013671875</v>
       </c>
       <c r="H4">
-        <v>45.37</v>
+        <v>79.47021484375</v>
       </c>
       <c r="I4">
-        <v>467.88009765625</v>
+        <v>494.669921875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1125,13 +1125,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>482.7998828125</v>
+        <v>559.669921875</v>
       </c>
       <c r="H5">
-        <v>43.17</v>
+        <v>81.56982421875</v>
       </c>
       <c r="I5">
-        <v>439.6298828125</v>
+        <v>478.10009765625</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Resultado final da rodada 8
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -52,12 +52,12 @@
     <t>Grupo I</t>
   </si>
   <si>
+    <t>JV5 Tricolor Gaúcho</t>
+  </si>
+  <si>
     <t>Bandoleros FCS</t>
   </si>
   <si>
-    <t>JV5 Tricolor Gaúcho</t>
-  </si>
-  <si>
     <t>LISI GREMISTA</t>
   </si>
   <si>
@@ -73,12 +73,12 @@
     <t>Dom Camillo68</t>
   </si>
   <si>
+    <t>A Lenda Super Vasco F.c</t>
+  </si>
+  <si>
     <t>Tatols Beants F.C</t>
   </si>
   <si>
-    <t>A Lenda Super Vasco F.c</t>
-  </si>
-  <si>
     <t>Grupo K</t>
   </si>
   <si>
@@ -88,22 +88,22 @@
     <t>TEAM LOPES 99</t>
   </si>
   <si>
+    <t>DM Studio</t>
+  </si>
+  <si>
     <t>TORRESMO COM PINGA PRO26.1</t>
   </si>
   <si>
-    <t>DM Studio</t>
-  </si>
-  <si>
     <t>Grupo L</t>
   </si>
   <si>
+    <t>Tabajara de Inhaua PB1</t>
+  </si>
+  <si>
+    <t>Texas Club 2026</t>
+  </si>
+  <si>
     <t>lsauer fc</t>
-  </si>
-  <si>
-    <t>Tabajara de Inhaua PB1</t>
-  </si>
-  <si>
-    <t>Texas Club 2026</t>
   </si>
   <si>
     <t>KillerColorado</t>
@@ -507,10 +507,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -519,13 +519,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>609.759765625</v>
+        <v>603.03955078125</v>
       </c>
       <c r="H2">
-        <v>79.919921875</v>
+        <v>149.22021484375</v>
       </c>
       <c r="I2">
-        <v>529.83984375</v>
+        <v>453.8193359375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -548,16 +548,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>522.98974609375</v>
+        <v>689.35986328125</v>
       </c>
       <c r="H3">
-        <v>76.97021484375</v>
+        <v>164.77001953125</v>
       </c>
       <c r="I3">
-        <v>446.01953125</v>
+        <v>524.58984375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -571,10 +571,10 @@
         <v>13</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>524.799560546875</v>
+        <v>609.649658203125</v>
       </c>
       <c r="H4">
-        <v>77.06982421875</v>
+        <v>156.669921875</v>
       </c>
       <c r="I4">
-        <v>447.729736328125</v>
+        <v>452.979736328125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -612,16 +612,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>519.91943359375</v>
+        <v>592.16943359375</v>
       </c>
       <c r="H5">
-        <v>82.3701171875</v>
+        <v>162.419921875</v>
       </c>
       <c r="I5">
-        <v>437.54931640625</v>
+        <v>429.74951171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -677,10 +677,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -689,13 +689,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>576.64013671875</v>
+        <v>653.09033203125</v>
       </c>
       <c r="H2">
-        <v>50.570068359375</v>
+        <v>105.610107421875</v>
       </c>
       <c r="I2">
-        <v>526.070068359375</v>
+        <v>547.480224609375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -718,16 +718,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>565.25</v>
+        <v>620.2900390625</v>
       </c>
       <c r="H3">
-        <v>87.009765625</v>
+        <v>163.4599609375</v>
       </c>
       <c r="I3">
-        <v>478.240234375</v>
+        <v>456.830078125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -741,10 +741,10 @@
         <v>18</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -753,13 +753,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>513.989990234375</v>
+        <v>572.43994140625</v>
       </c>
       <c r="H4">
-        <v>87.1201171875</v>
+        <v>155.8701171875</v>
       </c>
       <c r="I4">
-        <v>426.869873046875</v>
+        <v>416.56982421875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>493.2900390625</v>
+        <v>583.889892578125</v>
       </c>
       <c r="H5">
-        <v>85.97021484375</v>
+        <v>166.27001953125</v>
       </c>
       <c r="I5">
-        <v>407.31982421875</v>
+        <v>417.619873046875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -847,10 +847,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>580.4296875</v>
+        <v>686.2998046875</v>
       </c>
       <c r="H2">
-        <v>72.1201171875</v>
+        <v>152.8701171875</v>
       </c>
       <c r="I2">
-        <v>508.3095703125</v>
+        <v>533.4296875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -888,16 +888,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>552.56005859375</v>
+        <v>633.31005859375</v>
       </c>
       <c r="H3">
-        <v>70.47021484375</v>
+        <v>176.34033203125</v>
       </c>
       <c r="I3">
-        <v>482.08984375</v>
+        <v>456.9697265625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -911,10 +911,10 @@
         <v>23</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>537.07958984375</v>
+        <v>596.209716796875</v>
       </c>
       <c r="H4">
-        <v>71.3701171875</v>
+        <v>180.8203125</v>
       </c>
       <c r="I4">
-        <v>465.70947265625</v>
+        <v>415.389404296875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>508.159912109375</v>
+        <v>612.02978515625</v>
       </c>
       <c r="H5">
-        <v>105.8701171875</v>
+        <v>159.419921875</v>
       </c>
       <c r="I5">
-        <v>402.289794921875</v>
+        <v>452.60986328125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1017,10 +1017,10 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>553.780029296875</v>
+        <v>603.64990234375</v>
       </c>
       <c r="H2">
-        <v>73.81982421875</v>
+        <v>150.3203125</v>
       </c>
       <c r="I2">
-        <v>479.960205078125</v>
+        <v>453.32958984375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1058,16 +1058,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>523.10009765625</v>
+        <v>650.59033203125</v>
       </c>
       <c r="H3">
-        <v>76.97021484375</v>
+        <v>153.990234375</v>
       </c>
       <c r="I3">
-        <v>446.1298828125</v>
+        <v>496.60009765625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1081,10 +1081,10 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1093,13 +1093,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>574.14013671875</v>
+        <v>627.130126953125</v>
       </c>
       <c r="H4">
-        <v>79.47021484375</v>
+        <v>154.36962890625</v>
       </c>
       <c r="I4">
-        <v>494.669921875</v>
+        <v>472.760498046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1122,16 +1122,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>559.669921875</v>
+        <v>634.18994140625</v>
       </c>
       <c r="H5">
-        <v>81.56982421875</v>
+        <v>158.02001953125</v>
       </c>
       <c r="I5">
-        <v>478.10009765625</v>
+        <v>476.169921875</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Corrige pontuacoes finais da rodada 8
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -82,10 +82,10 @@
     <t>Grupo K</t>
   </si>
   <si>
+    <t>TEAM LOPES 99</t>
+  </si>
+  <si>
     <t>Fedato Futebol Clube</t>
-  </si>
-  <si>
-    <t>TEAM LOPES 99</t>
   </si>
   <si>
     <t>DM Studio</t>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>686.2998046875</v>
+        <v>633.31005859375</v>
       </c>
       <c r="H2">
-        <v>152.8701171875</v>
+        <v>147.3701171875</v>
       </c>
       <c r="I2">
-        <v>533.4296875</v>
+        <v>485.93994140625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -891,13 +891,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>633.31005859375</v>
+        <v>657.32958984375</v>
       </c>
       <c r="H3">
-        <v>176.34033203125</v>
+        <v>152.8701171875</v>
       </c>
       <c r="I3">
-        <v>456.9697265625</v>
+        <v>504.45947265625</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>

<commit_message>
Atualiza Parcias da Rodada 9
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -52,15 +52,15 @@
     <t>Grupo I</t>
   </si>
   <si>
+    <t>Bandoleros FCS</t>
+  </si>
+  <si>
+    <t>LISI GREMISTA</t>
+  </si>
+  <si>
     <t>JV5 Tricolor Gaúcho</t>
   </si>
   <si>
-    <t>Bandoleros FCS</t>
-  </si>
-  <si>
-    <t>LISI GREMISTA</t>
-  </si>
-  <si>
     <t>Mau Humor F.C.</t>
   </si>
   <si>
@@ -73,12 +73,12 @@
     <t>Dom Camillo68</t>
   </si>
   <si>
+    <t>Tatols Beants F.C</t>
+  </si>
+  <si>
     <t>A Lenda Super Vasco F.c</t>
   </si>
   <si>
-    <t>Tatols Beants F.C</t>
-  </si>
-  <si>
     <t>Grupo K</t>
   </si>
   <si>
@@ -88,22 +88,22 @@
     <t>Fedato Futebol Clube</t>
   </si>
   <si>
+    <t>TORRESMO COM PINGA PRO26.1</t>
+  </si>
+  <si>
     <t>DM Studio</t>
   </si>
   <si>
-    <t>TORRESMO COM PINGA PRO26.1</t>
-  </si>
-  <si>
     <t>Grupo L</t>
   </si>
   <si>
+    <t>lsauer fc</t>
+  </si>
+  <si>
     <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
     <t>Texas Club 2026</t>
-  </si>
-  <si>
-    <t>lsauer fc</t>
   </si>
   <si>
     <t>KillerColorado</t>
@@ -516,16 +516,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>603.03955078125</v>
+        <v>762.30986328125</v>
       </c>
       <c r="H2">
-        <v>149.22021484375</v>
+        <v>225.78001953125</v>
       </c>
       <c r="I2">
-        <v>453.8193359375</v>
+        <v>536.5298437500001</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -539,10 +539,10 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -551,13 +551,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>689.35986328125</v>
+        <v>695.7096582031249</v>
       </c>
       <c r="H3">
-        <v>164.77001953125</v>
+        <v>216.049921875</v>
       </c>
       <c r="I3">
-        <v>524.58984375</v>
+        <v>479.6597363281249</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -571,10 +571,10 @@
         <v>13</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>609.649658203125</v>
+        <v>664.04955078125</v>
       </c>
       <c r="H4">
-        <v>156.669921875</v>
+        <v>222.17021484375</v>
       </c>
       <c r="I4">
-        <v>452.979736328125</v>
+        <v>441.8793359375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -612,16 +612,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>592.16943359375</v>
+        <v>651.54943359375</v>
       </c>
       <c r="H5">
-        <v>162.419921875</v>
+        <v>248.479921875</v>
       </c>
       <c r="I5">
-        <v>429.74951171875</v>
+        <v>403.06951171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -686,16 +686,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>653.09033203125</v>
+        <v>739.54033203125</v>
       </c>
       <c r="H2">
-        <v>105.610107421875</v>
+        <v>197.750107421875</v>
       </c>
       <c r="I2">
-        <v>547.480224609375</v>
+        <v>541.7902246093751</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -709,10 +709,10 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -721,13 +721,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>620.2900390625</v>
+        <v>714.1700390625</v>
       </c>
       <c r="H3">
-        <v>163.4599609375</v>
+        <v>235.5399609375</v>
       </c>
       <c r="I3">
-        <v>456.830078125</v>
+        <v>478.630078125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -750,16 +750,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>572.43994140625</v>
+        <v>676.029892578125</v>
       </c>
       <c r="H4">
-        <v>155.8701171875</v>
+        <v>252.72001953125</v>
       </c>
       <c r="I4">
-        <v>416.56982421875</v>
+        <v>423.309873046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -773,10 +773,10 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -785,13 +785,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>583.889892578125</v>
+        <v>644.51994140625</v>
       </c>
       <c r="H5">
-        <v>166.27001953125</v>
+        <v>249.7501171875</v>
       </c>
       <c r="I5">
-        <v>417.619873046875</v>
+        <v>394.76982421875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -847,10 +847,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>633.31005859375</v>
+        <v>717.7500585937501</v>
       </c>
       <c r="H2">
-        <v>147.3701171875</v>
+        <v>225.7301171875</v>
       </c>
       <c r="I2">
-        <v>485.93994140625</v>
+        <v>492.01994140625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -888,16 +888,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>657.32958984375</v>
+        <v>738.7695898437501</v>
       </c>
       <c r="H3">
-        <v>152.8701171875</v>
+        <v>243.2501171875</v>
       </c>
       <c r="I3">
-        <v>504.45947265625</v>
+        <v>495.5194726562501</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -920,16 +920,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>596.209716796875</v>
+        <v>702.40978515625</v>
       </c>
       <c r="H4">
-        <v>180.8203125</v>
+        <v>240.859921875</v>
       </c>
       <c r="I4">
-        <v>415.389404296875</v>
+        <v>461.54986328125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -943,10 +943,10 @@
         <v>24</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -955,13 +955,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>612.02978515625</v>
+        <v>674.569716796875</v>
       </c>
       <c r="H5">
-        <v>159.419921875</v>
+        <v>265.2603125</v>
       </c>
       <c r="I5">
-        <v>452.60986328125</v>
+        <v>409.309404296875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1026,16 +1026,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>603.64990234375</v>
+        <v>731.8101269531251</v>
       </c>
       <c r="H2">
-        <v>150.3203125</v>
+        <v>240.81962890625</v>
       </c>
       <c r="I2">
-        <v>453.32958984375</v>
+        <v>490.9904980468751</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1049,10 +1049,10 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1061,13 +1061,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>650.59033203125</v>
+        <v>668.72990234375</v>
       </c>
       <c r="H3">
-        <v>153.990234375</v>
+        <v>235.1703125</v>
       </c>
       <c r="I3">
-        <v>496.60009765625</v>
+        <v>433.55958984375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>627.130126953125</v>
+        <v>737.04033203125</v>
       </c>
       <c r="H4">
-        <v>154.36962890625</v>
+        <v>258.670234375</v>
       </c>
       <c r="I4">
-        <v>472.760498046875</v>
+        <v>478.37009765625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1113,10 +1113,10 @@
         <v>29</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1125,13 +1125,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>634.18994140625</v>
+        <v>719.03994140625</v>
       </c>
       <c r="H5">
-        <v>158.02001953125</v>
+        <v>223.10001953125</v>
       </c>
       <c r="I5">
-        <v>476.169921875</v>
+        <v>495.939921875</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Resultado Final da Rodada 9
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -519,13 +519,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>762.30986328125</v>
+        <v>760.40966796875</v>
       </c>
       <c r="H2">
-        <v>225.78001953125</v>
+        <v>223.780029296875</v>
       </c>
       <c r="I2">
-        <v>536.5298437500001</v>
+        <v>536.629638671875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -551,13 +551,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>695.7096582031249</v>
+        <v>694.209716796875</v>
       </c>
       <c r="H3">
-        <v>216.049921875</v>
+        <v>216.0498046875</v>
       </c>
       <c r="I3">
-        <v>479.6597363281249</v>
+        <v>478.159912109375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>664.04955078125</v>
+        <v>662.049560546875</v>
       </c>
       <c r="H4">
-        <v>222.17021484375</v>
+        <v>220.27001953125</v>
       </c>
       <c r="I4">
-        <v>441.8793359375</v>
+        <v>441.779541015625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -615,13 +615,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>651.54943359375</v>
+        <v>651.54931640625</v>
       </c>
       <c r="H5">
-        <v>248.479921875</v>
+        <v>246.97998046875</v>
       </c>
       <c r="I5">
-        <v>403.06951171875</v>
+        <v>404.5693359375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -689,13 +689,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>739.54033203125</v>
+        <v>738.9404296875</v>
       </c>
       <c r="H2">
-        <v>197.750107421875</v>
+        <v>196.750244140625</v>
       </c>
       <c r="I2">
-        <v>541.7902246093751</v>
+        <v>542.190185546875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -721,13 +721,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>714.1700390625</v>
+        <v>714.169921875</v>
       </c>
       <c r="H3">
-        <v>235.5399609375</v>
+        <v>235.5400390625</v>
       </c>
       <c r="I3">
-        <v>478.630078125</v>
+        <v>478.6298828125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -753,13 +753,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>676.029892578125</v>
+        <v>675.030029296875</v>
       </c>
       <c r="H4">
-        <v>252.72001953125</v>
+        <v>252.1201171875</v>
       </c>
       <c r="I4">
-        <v>423.309873046875</v>
+        <v>422.909912109375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -785,13 +785,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>644.51994140625</v>
+        <v>644.52001953125</v>
       </c>
       <c r="H5">
-        <v>249.7501171875</v>
+        <v>249.75</v>
       </c>
       <c r="I5">
-        <v>394.76982421875</v>
+        <v>394.77001953125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>717.7500585937501</v>
+        <v>717.75</v>
       </c>
       <c r="H2">
-        <v>225.7301171875</v>
+        <v>225.72998046875</v>
       </c>
       <c r="I2">
-        <v>492.01994140625</v>
+        <v>492.02001953125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -891,13 +891,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>738.7695898437501</v>
+        <v>737.26953125</v>
       </c>
       <c r="H3">
-        <v>243.2501171875</v>
+        <v>243.25</v>
       </c>
       <c r="I3">
-        <v>495.5194726562501</v>
+        <v>494.01953125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -923,13 +923,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>702.40978515625</v>
+        <v>702.40966796875</v>
       </c>
       <c r="H4">
-        <v>240.859921875</v>
+        <v>239.35986328125</v>
       </c>
       <c r="I4">
-        <v>461.54986328125</v>
+        <v>463.0498046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -955,13 +955,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>674.569716796875</v>
+        <v>674.569580078125</v>
       </c>
       <c r="H5">
-        <v>265.2603125</v>
+        <v>265.26025390625</v>
       </c>
       <c r="I5">
-        <v>409.309404296875</v>
+        <v>409.309326171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1029,13 +1029,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>731.8101269531251</v>
+        <v>731.810302734375</v>
       </c>
       <c r="H2">
-        <v>240.81962890625</v>
+        <v>240.2197265625</v>
       </c>
       <c r="I2">
-        <v>490.9904980468751</v>
+        <v>491.590576171875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1061,13 +1061,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>668.72990234375</v>
+        <v>667.429931640625</v>
       </c>
       <c r="H3">
-        <v>235.1703125</v>
+        <v>234.5703125</v>
       </c>
       <c r="I3">
-        <v>433.55958984375</v>
+        <v>432.859619140625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1093,13 +1093,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>737.04033203125</v>
+        <v>736.4404296875</v>
       </c>
       <c r="H4">
-        <v>258.670234375</v>
+        <v>258.67041015625</v>
       </c>
       <c r="I4">
-        <v>478.37009765625</v>
+        <v>477.77001953125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1125,13 +1125,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>719.03994140625</v>
+        <v>718.43994140625</v>
       </c>
       <c r="H5">
-        <v>223.10001953125</v>
+        <v>221.800048828125</v>
       </c>
       <c r="I5">
-        <v>495.939921875</v>
+        <v>496.639892578125</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza Parciais da Rodada10
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -52,13 +52,13 @@
     <t>Grupo I</t>
   </si>
   <si>
+    <t>JV5 Tricolor Gaúcho</t>
+  </si>
+  <si>
     <t>Bandoleros FCS</t>
   </si>
   <si>
     <t>LISI GREMISTA</t>
-  </si>
-  <si>
-    <t>JV5 Tricolor Gaúcho</t>
   </si>
   <si>
     <t>Mau Humor F.C.</t>
@@ -507,10 +507,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -519,13 +519,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>760.40966796875</v>
+        <v>722.6195605468751</v>
       </c>
       <c r="H2">
-        <v>223.780029296875</v>
+        <v>278.74001953125</v>
       </c>
       <c r="I2">
-        <v>536.629638671875</v>
+        <v>443.879541015625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -548,16 +548,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>694.209716796875</v>
+        <v>818.29966796875</v>
       </c>
       <c r="H3">
-        <v>216.0498046875</v>
+        <v>290.450029296875</v>
       </c>
       <c r="I3">
-        <v>478.159912109375</v>
+        <v>527.849638671875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -580,16 +580,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>662.049560546875</v>
+        <v>752.679716796875</v>
       </c>
       <c r="H4">
-        <v>220.27001953125</v>
+        <v>276.6198046875</v>
       </c>
       <c r="I4">
-        <v>441.779541015625</v>
+        <v>476.059912109375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -603,10 +603,10 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -615,13 +615,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>651.54931640625</v>
+        <v>718.21931640625</v>
       </c>
       <c r="H5">
-        <v>246.97998046875</v>
+        <v>304.86998046875</v>
       </c>
       <c r="I5">
-        <v>404.5693359375</v>
+        <v>413.3493359375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -677,10 +677,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -689,13 +689,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>738.9404296875</v>
+        <v>798.2304296875</v>
       </c>
       <c r="H2">
-        <v>196.750244140625</v>
+        <v>245.920244140625</v>
       </c>
       <c r="I2">
-        <v>542.190185546875</v>
+        <v>552.3101855468749</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -709,10 +709,10 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -721,13 +721,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>714.169921875</v>
+        <v>766.139921875</v>
       </c>
       <c r="H3">
-        <v>235.5400390625</v>
+        <v>283.8100390625</v>
       </c>
       <c r="I3">
-        <v>478.6298828125</v>
+        <v>482.3298828125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -750,16 +750,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>675.030029296875</v>
+        <v>723.300029296875</v>
       </c>
       <c r="H4">
-        <v>252.1201171875</v>
+        <v>304.0901171875</v>
       </c>
       <c r="I4">
-        <v>422.909912109375</v>
+        <v>419.209912109375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>644.52001953125</v>
+        <v>693.69001953125</v>
       </c>
       <c r="H5">
-        <v>249.75</v>
+        <v>309.04</v>
       </c>
       <c r="I5">
-        <v>394.77001953125</v>
+        <v>384.6500195312499</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -847,10 +847,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>717.75</v>
+        <v>786.22</v>
       </c>
       <c r="H2">
-        <v>225.72998046875</v>
+        <v>284.11998046875</v>
       </c>
       <c r="I2">
-        <v>492.02001953125</v>
+        <v>502.10001953125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -879,10 +879,10 @@
         <v>22</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -891,13 +891,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>737.26953125</v>
+        <v>792.4595312500001</v>
       </c>
       <c r="H3">
-        <v>243.25</v>
+        <v>298.03</v>
       </c>
       <c r="I3">
-        <v>494.01953125</v>
+        <v>494.4295312500001</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -920,16 +920,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>702.40966796875</v>
+        <v>760.79966796875</v>
       </c>
       <c r="H4">
-        <v>239.35986328125</v>
+        <v>307.82986328125</v>
       </c>
       <c r="I4">
-        <v>463.0498046875</v>
+        <v>452.9698046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>674.569580078125</v>
+        <v>729.349580078125</v>
       </c>
       <c r="H5">
-        <v>265.26025390625</v>
+        <v>320.45025390625</v>
       </c>
       <c r="I5">
-        <v>409.309326171875</v>
+        <v>408.899326171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1017,10 +1017,10 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1029,13 +1029,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>731.810302734375</v>
+        <v>799.100302734375</v>
       </c>
       <c r="H2">
-        <v>240.2197265625</v>
+        <v>278.2097265625</v>
       </c>
       <c r="I2">
-        <v>491.590576171875</v>
+        <v>520.890576171875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1049,10 +1049,10 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1061,13 +1061,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>667.429931640625</v>
+        <v>732.1199316406251</v>
       </c>
       <c r="H3">
-        <v>234.5703125</v>
+        <v>293.8603125</v>
       </c>
       <c r="I3">
-        <v>432.859619140625</v>
+        <v>438.259619140625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>736.4404296875</v>
+        <v>795.7304296875</v>
       </c>
       <c r="H4">
-        <v>258.67041015625</v>
+        <v>323.36041015625</v>
       </c>
       <c r="I4">
-        <v>477.77001953125</v>
+        <v>472.37001953125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1122,16 +1122,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>718.43994140625</v>
+        <v>756.42994140625</v>
       </c>
       <c r="H5">
-        <v>221.800048828125</v>
+        <v>289.090048828125</v>
       </c>
       <c r="I5">
-        <v>496.639892578125</v>
+        <v>467.339892578125</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Resultado Final da Rodada 10
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -519,13 +519,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>722.6195605468751</v>
+        <v>722.219482421875</v>
       </c>
       <c r="H2">
-        <v>278.74001953125</v>
+        <v>278.340087890625</v>
       </c>
       <c r="I2">
-        <v>443.879541015625</v>
+        <v>443.87939453125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -551,13 +551,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>818.29966796875</v>
+        <v>817.899658203125</v>
       </c>
       <c r="H3">
-        <v>290.450029296875</v>
+        <v>290.050048828125</v>
       </c>
       <c r="I3">
-        <v>527.849638671875</v>
+        <v>527.849609375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -583,13 +583,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>752.679716796875</v>
+        <v>752.27978515625</v>
       </c>
       <c r="H4">
-        <v>276.6198046875</v>
+        <v>276.2197265625</v>
       </c>
       <c r="I4">
-        <v>476.059912109375</v>
+        <v>476.06005859375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -615,13 +615,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>718.21931640625</v>
+        <v>717.8193359375</v>
       </c>
       <c r="H5">
-        <v>304.86998046875</v>
+        <v>304.469970703125</v>
       </c>
       <c r="I5">
-        <v>413.3493359375</v>
+        <v>413.349365234375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -689,13 +689,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>798.2304296875</v>
+        <v>797.030517578125</v>
       </c>
       <c r="H2">
-        <v>245.920244140625</v>
+        <v>244.72021484375</v>
       </c>
       <c r="I2">
-        <v>552.3101855468749</v>
+        <v>552.310302734375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -721,13 +721,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>766.139921875</v>
+        <v>765.739990234375</v>
       </c>
       <c r="H3">
-        <v>283.8100390625</v>
+        <v>283.41015625</v>
       </c>
       <c r="I3">
-        <v>482.3298828125</v>
+        <v>482.329833984375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -753,13 +753,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>723.300029296875</v>
+        <v>722.900146484375</v>
       </c>
       <c r="H4">
-        <v>304.0901171875</v>
+        <v>303.690185546875</v>
       </c>
       <c r="I4">
-        <v>419.209912109375</v>
+        <v>419.2099609375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -785,13 +785,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>693.69001953125</v>
+        <v>692.489990234375</v>
       </c>
       <c r="H5">
-        <v>309.04</v>
+        <v>307.840087890625</v>
       </c>
       <c r="I5">
-        <v>384.6500195312499</v>
+        <v>384.64990234375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>786.22</v>
+        <v>785.02001953125</v>
       </c>
       <c r="H2">
-        <v>284.11998046875</v>
+        <v>282.919921875</v>
       </c>
       <c r="I2">
-        <v>502.10001953125</v>
+        <v>502.10009765625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -891,13 +891,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>792.4595312500001</v>
+        <v>791.659423828125</v>
       </c>
       <c r="H3">
-        <v>298.03</v>
+        <v>297.22998046875</v>
       </c>
       <c r="I3">
-        <v>494.4295312500001</v>
+        <v>494.429443359375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -923,13 +923,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>760.79966796875</v>
+        <v>759.599609375</v>
       </c>
       <c r="H4">
-        <v>307.82986328125</v>
+        <v>306.6298828125</v>
       </c>
       <c r="I4">
-        <v>452.9698046875</v>
+        <v>452.9697265625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -955,13 +955,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>729.349580078125</v>
+        <v>728.549560546875</v>
       </c>
       <c r="H5">
-        <v>320.45025390625</v>
+        <v>319.650146484375</v>
       </c>
       <c r="I5">
-        <v>408.899326171875</v>
+        <v>408.8994140625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1029,13 +1029,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>799.100302734375</v>
+        <v>798.700439453125</v>
       </c>
       <c r="H2">
-        <v>278.2097265625</v>
+        <v>277.40966796875</v>
       </c>
       <c r="I2">
-        <v>520.890576171875</v>
+        <v>521.290771484375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1061,13 +1061,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>732.1199316406251</v>
+        <v>731.719970703125</v>
       </c>
       <c r="H3">
-        <v>293.8603125</v>
+        <v>292.660400390625</v>
       </c>
       <c r="I3">
-        <v>438.259619140625</v>
+        <v>439.0595703125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1093,13 +1093,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>795.7304296875</v>
+        <v>794.530517578125</v>
       </c>
       <c r="H4">
-        <v>323.36041015625</v>
+        <v>322.96044921875</v>
       </c>
       <c r="I4">
-        <v>472.37001953125</v>
+        <v>471.570068359375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1125,13 +1125,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>756.42994140625</v>
+        <v>755.6298828125</v>
       </c>
       <c r="H5">
-        <v>289.090048828125</v>
+        <v>288.690185546875</v>
       </c>
       <c r="I5">
-        <v>467.339892578125</v>
+        <v>466.939697265625</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Resultado Final da Rodada 11
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -52,15 +52,15 @@
     <t>Grupo I</t>
   </si>
   <si>
+    <t>LISI GREMISTA</t>
+  </si>
+  <si>
     <t>JV5 Tricolor Gaúcho</t>
   </si>
   <si>
     <t>Bandoleros FCS</t>
   </si>
   <si>
-    <t>LISI GREMISTA</t>
-  </si>
-  <si>
     <t>Mau Humor F.C.</t>
   </si>
   <si>
@@ -73,12 +73,12 @@
     <t>Dom Camillo68</t>
   </si>
   <si>
+    <t>A Lenda Super Vasco F.c</t>
+  </si>
+  <si>
     <t>Tatols Beants F.C</t>
   </si>
   <si>
-    <t>A Lenda Super Vasco F.c</t>
-  </si>
-  <si>
     <t>Grupo K</t>
   </si>
   <si>
@@ -88,12 +88,12 @@
     <t>Fedato Futebol Clube</t>
   </si>
   <si>
+    <t>DM Studio</t>
+  </si>
+  <si>
     <t>TORRESMO COM PINGA PRO26.1</t>
   </si>
   <si>
-    <t>DM Studio</t>
-  </si>
-  <si>
     <t>Grupo L</t>
   </si>
   <si>
@@ -103,10 +103,10 @@
     <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
+    <t>KillerColorado</t>
+  </si>
+  <si>
     <t>Texas Club 2026</t>
-  </si>
-  <si>
-    <t>KillerColorado</t>
   </si>
 </sst>
 </file>
@@ -516,16 +516,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>722.219482421875</v>
+        <v>844.83984375</v>
       </c>
       <c r="H2">
-        <v>278.340087890625</v>
+        <v>346.3798828125</v>
       </c>
       <c r="I2">
-        <v>443.87939453125</v>
+        <v>498.4599609375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -539,10 +539,10 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -551,13 +551,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>817.899658203125</v>
+        <v>805.029541015625</v>
       </c>
       <c r="H3">
-        <v>290.050048828125</v>
+        <v>384.300048828125</v>
       </c>
       <c r="I3">
-        <v>527.849609375</v>
+        <v>420.7294921875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -580,16 +580,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>752.27978515625</v>
+        <v>888.059814453125</v>
       </c>
       <c r="H4">
-        <v>276.2197265625</v>
+        <v>382.610107421875</v>
       </c>
       <c r="I4">
-        <v>476.06005859375</v>
+        <v>505.44970703125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -603,10 +603,10 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -615,13 +615,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>717.8193359375</v>
+        <v>823.779296875</v>
       </c>
       <c r="H5">
-        <v>304.469970703125</v>
+        <v>387.280029296875</v>
       </c>
       <c r="I5">
-        <v>413.349365234375</v>
+        <v>436.499267578125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -677,10 +677,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -689,13 +689,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>797.030517578125</v>
+        <v>876.690673828125</v>
       </c>
       <c r="H2">
-        <v>244.72021484375</v>
+        <v>324.30029296875</v>
       </c>
       <c r="I2">
-        <v>552.310302734375</v>
+        <v>552.390380859375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -718,16 +718,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>765.739990234375</v>
+        <v>845.320068359375</v>
       </c>
       <c r="H3">
-        <v>283.41015625</v>
+        <v>363.0703125</v>
       </c>
       <c r="I3">
-        <v>482.329833984375</v>
+        <v>482.249755859375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -741,10 +741,10 @@
         <v>18</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -753,13 +753,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>722.900146484375</v>
+        <v>779.949951171875</v>
       </c>
       <c r="H4">
-        <v>303.690185546875</v>
+        <v>391.320068359375</v>
       </c>
       <c r="I4">
-        <v>419.2099609375</v>
+        <v>388.6298828125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>692.489990234375</v>
+        <v>806.380126953125</v>
       </c>
       <c r="H5">
-        <v>307.840087890625</v>
+        <v>391.150146484375</v>
       </c>
       <c r="I5">
-        <v>384.64990234375</v>
+        <v>415.22998046875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -847,10 +847,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>785.02001953125</v>
+        <v>879.080078125</v>
       </c>
       <c r="H2">
-        <v>282.919921875</v>
+        <v>374.19970703125</v>
       </c>
       <c r="I2">
-        <v>502.10009765625</v>
+        <v>504.88037109375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -888,16 +888,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>791.659423828125</v>
+        <v>882.939208984375</v>
       </c>
       <c r="H3">
-        <v>297.22998046875</v>
+        <v>391.2900390625</v>
       </c>
       <c r="I3">
-        <v>494.429443359375</v>
+        <v>491.649169921875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -911,10 +911,10 @@
         <v>23</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>759.599609375</v>
+        <v>816.309326171875</v>
       </c>
       <c r="H4">
-        <v>306.6298828125</v>
+        <v>405.909912109375</v>
       </c>
       <c r="I4">
-        <v>452.9697265625</v>
+        <v>410.3994140625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>728.549560546875</v>
+        <v>845.859375</v>
       </c>
       <c r="H5">
-        <v>319.650146484375</v>
+        <v>394.3896484375</v>
       </c>
       <c r="I5">
-        <v>408.8994140625</v>
+        <v>451.4697265625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1017,10 +1017,10 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1029,13 +1029,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>798.700439453125</v>
+        <v>889.160400390625</v>
       </c>
       <c r="H2">
-        <v>277.40966796875</v>
+        <v>359.16943359375</v>
       </c>
       <c r="I2">
-        <v>521.290771484375</v>
+        <v>529.990966796875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1058,16 +1058,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>731.719970703125</v>
+        <v>813.479736328125</v>
       </c>
       <c r="H3">
-        <v>292.660400390625</v>
+        <v>383.120361328125</v>
       </c>
       <c r="I3">
-        <v>439.0595703125</v>
+        <v>430.359375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1081,10 +1081,10 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1093,13 +1093,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>794.530517578125</v>
+        <v>870.8896484375</v>
       </c>
       <c r="H4">
-        <v>322.96044921875</v>
+        <v>377.449951171875</v>
       </c>
       <c r="I4">
-        <v>471.570068359375</v>
+        <v>493.439697265625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1122,16 +1122,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>755.6298828125</v>
+        <v>883.290283203125</v>
       </c>
       <c r="H5">
-        <v>288.690185546875</v>
+        <v>438.22021484375</v>
       </c>
       <c r="I5">
-        <v>466.939697265625</v>
+        <v>445.070068359375</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza Parciais da Rodada 12
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -52,18 +52,18 @@
     <t>Grupo I</t>
   </si>
   <si>
+    <t>Bandoleros FCS</t>
+  </si>
+  <si>
     <t>LISI GREMISTA</t>
   </si>
   <si>
+    <t>Mau Humor F.C.</t>
+  </si>
+  <si>
     <t>JV5 Tricolor Gaúcho</t>
   </si>
   <si>
-    <t>Bandoleros FCS</t>
-  </si>
-  <si>
-    <t>Mau Humor F.C.</t>
-  </si>
-  <si>
     <t>Grupo J</t>
   </si>
   <si>
@@ -88,12 +88,12 @@
     <t>Fedato Futebol Clube</t>
   </si>
   <si>
+    <t>TORRESMO COM PINGA PRO26.1</t>
+  </si>
+  <si>
     <t>DM Studio</t>
   </si>
   <si>
-    <t>TORRESMO COM PINGA PRO26.1</t>
-  </si>
-  <si>
     <t>Grupo L</t>
   </si>
   <si>
@@ -103,10 +103,10 @@
     <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
+    <t>Texas Club 2026</t>
+  </si>
+  <si>
     <t>KillerColorado</t>
-  </si>
-  <si>
-    <t>Texas Club 2026</t>
   </si>
 </sst>
 </file>
@@ -516,16 +516,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>844.83984375</v>
+        <v>971.759814453125</v>
       </c>
       <c r="H2">
-        <v>346.3798828125</v>
+        <v>459.960107421875</v>
       </c>
       <c r="I2">
-        <v>498.4599609375</v>
+        <v>511.79970703125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -548,16 +548,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>805.029541015625</v>
+        <v>915.43984375</v>
       </c>
       <c r="H3">
-        <v>384.300048828125</v>
+        <v>423.6298828125</v>
       </c>
       <c r="I3">
-        <v>420.7294921875</v>
+        <v>491.8099609375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -571,10 +571,10 @@
         <v>13</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>888.059814453125</v>
+        <v>901.029296875</v>
       </c>
       <c r="H4">
-        <v>382.610107421875</v>
+        <v>457.880029296875</v>
       </c>
       <c r="I4">
-        <v>505.44970703125</v>
+        <v>443.149267578125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -603,10 +603,10 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -615,13 +615,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>823.779296875</v>
+        <v>882.379541015625</v>
       </c>
       <c r="H5">
-        <v>387.280029296875</v>
+        <v>468.000048828125</v>
       </c>
       <c r="I5">
-        <v>436.499267578125</v>
+        <v>414.3794921875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -677,10 +677,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -689,13 +689,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>876.690673828125</v>
+        <v>961.090673828125</v>
       </c>
       <c r="H2">
-        <v>324.30029296875</v>
+        <v>388.10029296875</v>
       </c>
       <c r="I2">
-        <v>552.390380859375</v>
+        <v>572.9903808593749</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -709,10 +709,10 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -721,13 +721,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>845.320068359375</v>
+        <v>923.270068359375</v>
       </c>
       <c r="H3">
-        <v>363.0703125</v>
+        <v>432.8703125</v>
       </c>
       <c r="I3">
-        <v>482.249755859375</v>
+        <v>490.399755859375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -750,16 +750,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>779.949951171875</v>
+        <v>849.749951171875</v>
       </c>
       <c r="H4">
-        <v>391.320068359375</v>
+        <v>469.270068359375</v>
       </c>
       <c r="I4">
-        <v>388.6298828125</v>
+        <v>380.4798828125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>806.380126953125</v>
+        <v>870.180126953125</v>
       </c>
       <c r="H5">
-        <v>391.150146484375</v>
+        <v>475.550146484375</v>
       </c>
       <c r="I5">
-        <v>415.22998046875</v>
+        <v>394.62998046875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -847,10 +847,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>879.080078125</v>
+        <v>963.580078125</v>
       </c>
       <c r="H2">
-        <v>374.19970703125</v>
+        <v>450.94970703125</v>
       </c>
       <c r="I2">
-        <v>504.88037109375</v>
+        <v>512.63037109375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -888,16 +888,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>882.939208984375</v>
+        <v>964.039208984375</v>
       </c>
       <c r="H3">
-        <v>391.2900390625</v>
+        <v>474.1900390625</v>
       </c>
       <c r="I3">
-        <v>491.649169921875</v>
+        <v>489.849169921875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -920,16 +920,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>816.309326171875</v>
+        <v>928.759375</v>
       </c>
       <c r="H4">
-        <v>405.909912109375</v>
+        <v>475.4896484375</v>
       </c>
       <c r="I4">
-        <v>410.3994140625</v>
+        <v>453.2697265625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -943,10 +943,10 @@
         <v>24</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -955,13 +955,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>845.859375</v>
+        <v>893.059326171875</v>
       </c>
       <c r="H5">
-        <v>394.3896484375</v>
+        <v>490.409912109375</v>
       </c>
       <c r="I5">
-        <v>451.4697265625</v>
+        <v>402.6494140625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1026,16 +1026,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>889.160400390625</v>
+        <v>973.560400390625</v>
       </c>
       <c r="H2">
-        <v>359.16943359375</v>
+        <v>445.82943359375</v>
       </c>
       <c r="I2">
-        <v>529.990966796875</v>
+        <v>527.730966796875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1049,10 +1049,10 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1061,13 +1061,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>813.479736328125</v>
+        <v>887.879736328125</v>
       </c>
       <c r="H3">
-        <v>383.120361328125</v>
+        <v>447.600361328125</v>
       </c>
       <c r="I3">
-        <v>430.359375</v>
+        <v>440.279375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>870.8896484375</v>
+        <v>969.950283203125</v>
       </c>
       <c r="H4">
-        <v>377.449951171875</v>
+        <v>522.62021484375</v>
       </c>
       <c r="I4">
-        <v>493.439697265625</v>
+        <v>447.330068359375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1113,10 +1113,10 @@
         <v>29</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1125,13 +1125,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>883.290283203125</v>
+        <v>935.3696484375</v>
       </c>
       <c r="H5">
-        <v>438.22021484375</v>
+        <v>451.849951171875</v>
       </c>
       <c r="I5">
-        <v>445.070068359375</v>
+        <v>483.519697265625</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Organiza terceiros e quartos colocados da fase 2 da Libertadores
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -519,13 +519,13 @@
         <v>3</v>
       </c>
       <c r="G2">
-        <v>971.759814453125</v>
+        <v>885.339892578125</v>
       </c>
       <c r="H2">
         <v>459.960107421875</v>
       </c>
       <c r="I2">
-        <v>511.79970703125</v>
+        <v>425.37978515625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -551,13 +551,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>915.43984375</v>
+        <v>851.07998046875</v>
       </c>
       <c r="H3">
         <v>423.6298828125</v>
       </c>
       <c r="I3">
-        <v>491.8099609375</v>
+        <v>427.45009765625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -583,13 +583,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>901.029296875</v>
+        <v>846.21923828125</v>
       </c>
       <c r="H4">
         <v>457.880029296875</v>
       </c>
       <c r="I4">
-        <v>443.149267578125</v>
+        <v>388.339208984375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -615,13 +615,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>882.379541015625</v>
+        <v>820.36953125</v>
       </c>
       <c r="H5">
         <v>468.000048828125</v>
       </c>
       <c r="I5">
-        <v>414.3794921875</v>
+        <v>352.369482421875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -689,13 +689,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>961.090673828125</v>
+        <v>878.090673828125</v>
       </c>
       <c r="H2">
         <v>388.10029296875</v>
       </c>
       <c r="I2">
-        <v>572.9903808593749</v>
+        <v>489.990380859375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -721,13 +721,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>923.270068359375</v>
+        <v>851.160205078125</v>
       </c>
       <c r="H3">
         <v>432.8703125</v>
       </c>
       <c r="I3">
-        <v>490.399755859375</v>
+        <v>418.289892578125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -753,13 +753,13 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>849.749951171875</v>
+        <v>780.950146484375</v>
       </c>
       <c r="H4">
         <v>469.270068359375</v>
       </c>
       <c r="I4">
-        <v>380.4798828125</v>
+        <v>311.680078125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -785,13 +785,13 @@
         <v>5</v>
       </c>
       <c r="G5">
-        <v>870.180126953125</v>
+        <v>807.260205078125</v>
       </c>
       <c r="H5">
         <v>475.550146484375</v>
       </c>
       <c r="I5">
-        <v>394.62998046875</v>
+        <v>331.71005859375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -859,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>963.580078125</v>
+        <v>886.169921875</v>
       </c>
       <c r="H2">
         <v>450.94970703125</v>
       </c>
       <c r="I2">
-        <v>512.63037109375</v>
+        <v>435.22021484375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -891,13 +891,13 @@
         <v>4</v>
       </c>
       <c r="G3">
-        <v>964.039208984375</v>
+        <v>901.229150390625</v>
       </c>
       <c r="H3">
         <v>474.1900390625</v>
       </c>
       <c r="I3">
-        <v>489.849169921875</v>
+        <v>427.039111328125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -923,13 +923,13 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>928.759375</v>
+        <v>859.339453125</v>
       </c>
       <c r="H4">
         <v>475.4896484375</v>
       </c>
       <c r="I4">
-        <v>453.2697265625</v>
+        <v>383.8498046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -955,13 +955,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>893.059326171875</v>
+        <v>825.869384765625</v>
       </c>
       <c r="H5">
         <v>490.409912109375</v>
       </c>
       <c r="I5">
-        <v>402.6494140625</v>
+        <v>335.45947265625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1029,13 +1029,13 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>973.560400390625</v>
+        <v>914.95029296875</v>
       </c>
       <c r="H2">
         <v>445.82943359375</v>
       </c>
       <c r="I2">
-        <v>527.730966796875</v>
+        <v>469.120859375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1061,13 +1061,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>887.879736328125</v>
+        <v>818.759619140625</v>
       </c>
       <c r="H3">
         <v>447.600361328125</v>
       </c>
       <c r="I3">
-        <v>440.279375</v>
+        <v>371.1592578125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1093,13 +1093,13 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>969.950283203125</v>
+        <v>886.950283203125</v>
       </c>
       <c r="H4">
         <v>522.62021484375</v>
       </c>
       <c r="I4">
-        <v>447.330068359375</v>
+        <v>364.330068359375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1125,13 +1125,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>935.3696484375</v>
+        <v>869.47951171875</v>
       </c>
       <c r="H5">
         <v>451.849951171875</v>
       </c>
       <c r="I5">
-        <v>483.519697265625</v>
+        <v>417.629560546875</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Resultado Final Rodada 12
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -100,13 +100,13 @@
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>KillerColorado</t>
+  </si>
+  <si>
     <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
     <t>Texas Club 2026</t>
-  </si>
-  <si>
-    <t>KillerColorado</t>
   </si>
 </sst>
 </file>
@@ -519,13 +519,13 @@
         <v>3</v>
       </c>
       <c r="G2">
-        <v>971.759814453125</v>
+        <v>971.760009765625</v>
       </c>
       <c r="H2">
-        <v>459.960107421875</v>
+        <v>459.960205078125</v>
       </c>
       <c r="I2">
-        <v>511.79970703125</v>
+        <v>511.7998046875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -551,13 +551,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>915.43984375</v>
+        <v>915.43994140625</v>
       </c>
       <c r="H3">
         <v>423.6298828125</v>
       </c>
       <c r="I3">
-        <v>491.8099609375</v>
+        <v>491.81005859375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -586,10 +586,10 @@
         <v>901.029296875</v>
       </c>
       <c r="H4">
-        <v>457.880029296875</v>
+        <v>457.880126953125</v>
       </c>
       <c r="I4">
-        <v>443.149267578125</v>
+        <v>443.149169921875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -615,13 +615,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>882.379541015625</v>
+        <v>882.379638671875</v>
       </c>
       <c r="H5">
-        <v>468.000048828125</v>
+        <v>468.000244140625</v>
       </c>
       <c r="I5">
-        <v>414.3794921875</v>
+        <v>414.37939453125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -689,13 +689,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>961.090673828125</v>
+        <v>961.090576171875</v>
       </c>
       <c r="H2">
-        <v>388.10029296875</v>
+        <v>388.100341796875</v>
       </c>
       <c r="I2">
-        <v>572.9903808593749</v>
+        <v>572.990234375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -721,13 +721,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>923.270068359375</v>
+        <v>923.270263671875</v>
       </c>
       <c r="H3">
-        <v>432.8703125</v>
+        <v>432.8701171875</v>
       </c>
       <c r="I3">
-        <v>490.399755859375</v>
+        <v>490.400146484375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -753,13 +753,13 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>849.749951171875</v>
+        <v>849.749755859375</v>
       </c>
       <c r="H4">
-        <v>469.270068359375</v>
+        <v>469.270263671875</v>
       </c>
       <c r="I4">
-        <v>380.4798828125</v>
+        <v>380.4794921875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -785,13 +785,13 @@
         <v>5</v>
       </c>
       <c r="G5">
-        <v>870.180126953125</v>
+        <v>870.18017578125</v>
       </c>
       <c r="H5">
-        <v>475.550146484375</v>
+        <v>475.550048828125</v>
       </c>
       <c r="I5">
-        <v>394.62998046875</v>
+        <v>394.630126953125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -891,13 +891,13 @@
         <v>4</v>
       </c>
       <c r="G3">
-        <v>964.039208984375</v>
+        <v>964.039306640625</v>
       </c>
       <c r="H3">
-        <v>474.1900390625</v>
+        <v>474.18994140625</v>
       </c>
       <c r="I3">
-        <v>489.849169921875</v>
+        <v>489.849365234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -923,13 +923,13 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>928.759375</v>
+        <v>928.75927734375</v>
       </c>
       <c r="H4">
-        <v>475.4896484375</v>
+        <v>475.48974609375</v>
       </c>
       <c r="I4">
-        <v>453.2697265625</v>
+        <v>453.26953125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1029,13 +1029,13 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>973.560400390625</v>
+        <v>973.560302734375</v>
       </c>
       <c r="H2">
-        <v>445.82943359375</v>
+        <v>445.82958984375</v>
       </c>
       <c r="I2">
-        <v>527.730966796875</v>
+        <v>527.730712890625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1049,25 +1049,25 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>887.879736328125</v>
+        <v>986.1494140625</v>
       </c>
       <c r="H3">
-        <v>447.600361328125</v>
+        <v>451.849853515625</v>
       </c>
       <c r="I3">
-        <v>440.279375</v>
+        <v>534.299560546875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1081,25 +1081,25 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>969.950283203125</v>
+        <v>887.879638671875</v>
       </c>
       <c r="H4">
-        <v>522.62021484375</v>
+        <v>498.380126953125</v>
       </c>
       <c r="I4">
-        <v>447.330068359375</v>
+        <v>389.49951171875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1125,13 +1125,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>935.3696484375</v>
+        <v>969.950439453125</v>
       </c>
       <c r="H5">
-        <v>451.849951171875</v>
+        <v>522.6201171875</v>
       </c>
       <c r="I5">
-        <v>483.519697265625</v>
+        <v>447.330322265625</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Corrige pontuacoes da fase 2 da Libertadores
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_2.xlsx
@@ -100,13 +100,13 @@
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>Tabajara de Inhaua PB1</t>
+  </si>
+  <si>
+    <t>Texas Club 2026</t>
+  </si>
+  <si>
     <t>KillerColorado</t>
-  </si>
-  <si>
-    <t>Tabajara de Inhaua PB1</t>
-  </si>
-  <si>
-    <t>Texas Club 2026</t>
   </si>
 </sst>
 </file>
@@ -1049,25 +1049,25 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>986.1494140625</v>
+        <v>887.879638671875</v>
       </c>
       <c r="H3">
-        <v>451.849853515625</v>
+        <v>447.600341796875</v>
       </c>
       <c r="I3">
-        <v>534.299560546875</v>
+        <v>440.279296875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1081,25 +1081,25 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>887.879638671875</v>
+        <v>969.950439453125</v>
       </c>
       <c r="H4">
-        <v>498.380126953125</v>
+        <v>522.6201171875</v>
       </c>
       <c r="I4">
-        <v>389.49951171875</v>
+        <v>447.330322265625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1125,13 +1125,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>969.950439453125</v>
+        <v>935.36962890625</v>
       </c>
       <c r="H5">
-        <v>522.6201171875</v>
+        <v>451.849853515625</v>
       </c>
       <c r="I5">
-        <v>447.330322265625</v>
+        <v>483.519775390625</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>